<commit_message>
feat(qol): meals state the level of the buff they give
meals state the level of the buff they give, read from the program
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_food_text.xlsx
+++ b/mod_project/data_tables/qol_food_text.xlsx
@@ -584,7 +584,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Heal status ailments + 50% HP + gain Sun Veil.</t>
+          <t>Heal status ailments + 50% HP + gain Sun Veil Lv5.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -617,7 +617,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Heal status ailments + 50% HP and 40% TP + gain Water Enchant.</t>
+          <t>Heal status ailments + 50% HP and 40% TP + gain Water Enchant Lv5.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -650,7 +650,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Heal all TP + gain Divine Shield.</t>
+          <t>Heal all TP + gain Divine Shield Lv5.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -683,7 +683,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Heal status ailments + 80% HP and TP + gain Aim.</t>
+          <t>Heal status ailments + 80% HP and TP + gain Aim Lv10.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -716,7 +716,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Heal all HP and TP + gain Protect and Accelerator.</t>
+          <t>Heal all HP and TP + gain Protect Lv5 and Accelerator Lv5.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -782,7 +782,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Heal 30% TP + gain Fire Enchant.</t>
+          <t>Heal 30% TP + gain Fire Enchant Lv5.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -881,7 +881,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Heal status ailments + 60% HP and TP + gain Brave.</t>
+          <t>Heal status ailments + 60% HP and TP + gain Brave Lv5.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -914,7 +914,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Heal all HP + gain Protect and Fleet Foot.</t>
+          <t>Heal all HP + gain Protect Lv5 and Fleet Foot Lv10.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -947,7 +947,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Heal 80% HP and TP + gain Stab, Slash, and Bash Guard.</t>
+          <t>Heal 80% HP and TP + gain Stab, Slash, and Bash Guard Lv5.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -980,7 +980,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Heal status ailments + all HP and TP + gain Insurance.</t>
+          <t>Heal status ailments + all HP and TP + gain Insurance Lv5.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>

</xml_diff>